<commit_message>
add plotting functionality, island detection and fixes issue #48 and 49
</commit_message>
<xml_diff>
--- a/test/inputs/case39/case39.xlsx
+++ b/test/inputs/case39/case39.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nomyk\Desktop\Network Reduction Model\NetworkReduction.jl\test\inputs\case39\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{254E094D-4C92-47F4-B2DD-094E93ABDAC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC762E08-7933-4D41-BE06-667FEB243A30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lines" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="79">
   <si>
     <t>Line_name</t>
   </si>
@@ -262,6 +262,9 @@
   </si>
   <si>
     <t>Z</t>
+  </si>
+  <si>
+    <t>IsRepresentative</t>
   </si>
 </sst>
 </file>
@@ -1813,106 +1816,109 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E83B6B-55F4-43BC-99E9-09E10DB244FC}">
-  <dimension ref="A1:O40"/>
+  <dimension ref="A1:P40"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="15.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:16">
       <c r="A1" s="9" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="N1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="P1" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:16">
       <c r="A2" t="s">
         <v>36</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
       <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
         <v>97.6</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>44.2</v>
       </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
       <c r="F2">
         <v>0</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
         <v>77</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>1.0393836000000001</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>-13.536602</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>345</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>75</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>1.06</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>0.94</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:16">
       <c r="A3" t="s">
         <v>37</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
       <c r="C3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -1923,119 +1929,119 @@
       <c r="F3">
         <v>0</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
         <v>77</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>1.0484941000000001</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>-9.7852665999999999</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>345</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>75</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>1.06</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>0.94</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:16">
       <c r="A4" t="s">
         <v>38</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
       <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
         <v>322</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>2.4</v>
       </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
       <c r="F4">
         <v>0</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s">
         <v>77</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>1.0307077</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>-12.276384</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>345</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>8</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>1.06</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>0.94</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:16">
       <c r="A5" t="s">
         <v>39</v>
       </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
       <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
         <v>500</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>184</v>
       </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
       <c r="F5">
         <v>0</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="s">
         <v>77</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>1.0044599999999999</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>-12.626734000000001</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>345</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>8</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <v>1.06</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>0.94</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:16">
       <c r="A6" t="s">
         <v>40</v>
       </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
       <c r="C6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -2046,37 +2052,37 @@
       <c r="F6">
         <v>0</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
         <v>77</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>1.0060062999999999</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>-11.192339</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>345</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>8</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>1.06</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>0.94</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:16">
       <c r="A7" t="s">
         <v>41</v>
       </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
       <c r="C7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -2087,160 +2093,160 @@
       <c r="F7">
         <v>0</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
         <v>77</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>1.0082256000000001</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>-10.408329999999999</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>345</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>75</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>1.06</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>0.94</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:16">
       <c r="A8" t="s">
         <v>42</v>
       </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
       <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
         <v>233.8</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>84</v>
       </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
       <c r="F8">
         <v>0</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
         <v>77</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>0.99839728000000005</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>-12.755625999999999</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>345</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>75</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <v>1.06</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>0.94</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:16">
       <c r="A9" t="s">
         <v>43</v>
       </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
       <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
         <v>522</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>176.6</v>
       </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
       <c r="F9">
         <v>0</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
         <v>77</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>0.99787232000000003</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>-13.335844</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>345</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>75</v>
       </c>
-      <c r="L9">
+      <c r="M9">
         <v>1.06</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>0.94</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:16">
       <c r="A10" t="s">
         <v>44</v>
       </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
       <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
         <v>6.5</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>-66.599999999999994</v>
       </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
       <c r="F10">
         <v>0</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" t="s">
         <v>77</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>1.038332</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>-14.178442</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>345</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>75</v>
       </c>
-      <c r="L10">
+      <c r="M10">
         <v>1.06</v>
       </c>
-      <c r="M10">
+      <c r="N10">
         <v>0.94</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:16">
       <c r="A11" t="s">
         <v>45</v>
       </c>
-      <c r="B11">
-        <v>1</v>
-      </c>
       <c r="C11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -2251,37 +2257,37 @@
       <c r="F11">
         <v>0</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
         <v>77</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>1.0178430999999999</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>-8.1708750000000006</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>345</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>75</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <v>1.06</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <v>0.94</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:16">
       <c r="A12" t="s">
         <v>46</v>
       </c>
-      <c r="B12">
-        <v>1</v>
-      </c>
       <c r="C12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -2292,78 +2298,78 @@
       <c r="F12">
         <v>0</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12" t="s">
         <v>77</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>1.0133858</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>-8.9369662999999999</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>345</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>75</v>
       </c>
-      <c r="L12">
+      <c r="M12">
         <v>1.06</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <v>0.94</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:16">
       <c r="A13" t="s">
         <v>47</v>
       </c>
-      <c r="B13">
-        <v>1</v>
-      </c>
       <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
         <v>8.5299999999999994</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>88</v>
       </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
       <c r="F13">
         <v>0</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13" t="s">
         <v>77</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>1.000815</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>-8.9988235999999997</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>345</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>75</v>
       </c>
-      <c r="L13">
+      <c r="M13">
         <v>1.06</v>
       </c>
-      <c r="M13">
+      <c r="N13">
         <v>0.94</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:16">
       <c r="A14" t="s">
         <v>48</v>
       </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
       <c r="C14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -2374,37 +2380,37 @@
       <c r="F14">
         <v>0</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14" t="s">
         <v>77</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>1.014923</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>-8.9299271999999998</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>345</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>75</v>
       </c>
-      <c r="L14">
+      <c r="M14">
         <v>1.06</v>
       </c>
-      <c r="M14">
+      <c r="N14">
         <v>0.94</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:16">
       <c r="A15" t="s">
         <v>49</v>
       </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
       <c r="C15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -2415,119 +2421,119 @@
       <c r="F15">
         <v>0</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15" t="s">
         <v>77</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <v>1.012319</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <v>-10.715294999999999</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>345</v>
       </c>
-      <c r="K15" t="s">
+      <c r="L15" t="s">
         <v>75</v>
       </c>
-      <c r="L15">
+      <c r="M15">
         <v>1.06</v>
       </c>
-      <c r="M15">
+      <c r="N15">
         <v>0.94</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:16">
       <c r="A16" t="s">
         <v>50</v>
       </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
       <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
         <v>320</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>153</v>
       </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
       <c r="F16">
         <v>0</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16" t="s">
         <v>77</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>1.0161853999999999</v>
       </c>
-      <c r="I16">
+      <c r="J16">
         <v>-11.345399</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>345</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>76</v>
       </c>
-      <c r="L16">
+      <c r="M16">
         <v>1.06</v>
       </c>
-      <c r="M16">
+      <c r="N16">
         <v>0.94</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:14">
       <c r="A17" t="s">
         <v>51</v>
       </c>
-      <c r="B17">
-        <v>1</v>
-      </c>
       <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
         <v>329</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>32.299999999999997</v>
       </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
       <c r="F17">
         <v>0</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17" t="s">
         <v>77</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <v>1.0325203000000001</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <v>-10.033348</v>
       </c>
-      <c r="J17">
+      <c r="K17">
         <v>345</v>
       </c>
-      <c r="K17" t="s">
+      <c r="L17" t="s">
         <v>76</v>
       </c>
-      <c r="L17">
+      <c r="M17">
         <v>1.06</v>
       </c>
-      <c r="M17">
+      <c r="N17">
         <v>0.94</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:14">
       <c r="A18" t="s">
         <v>52</v>
       </c>
-      <c r="B18">
-        <v>1</v>
-      </c>
       <c r="C18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -2538,78 +2544,78 @@
       <c r="F18">
         <v>0</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
         <v>77</v>
       </c>
-      <c r="H18">
+      <c r="I18">
         <v>1.0342365</v>
       </c>
-      <c r="I18">
+      <c r="J18">
         <v>-11.116436</v>
       </c>
-      <c r="J18">
+      <c r="K18">
         <v>345</v>
       </c>
-      <c r="K18" t="s">
+      <c r="L18" t="s">
         <v>8</v>
       </c>
-      <c r="L18">
+      <c r="M18">
         <v>1.06</v>
       </c>
-      <c r="M18">
+      <c r="N18">
         <v>0.94</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:14">
       <c r="A19" t="s">
         <v>53</v>
       </c>
-      <c r="B19">
-        <v>1</v>
-      </c>
       <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
         <v>158</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>30</v>
       </c>
-      <c r="E19">
-        <v>0</v>
-      </c>
       <c r="F19">
         <v>0</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19" t="s">
         <v>77</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <v>1.0315726000000001</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <v>-11.986167999999999</v>
       </c>
-      <c r="J19">
+      <c r="K19">
         <v>345</v>
       </c>
-      <c r="K19" t="s">
+      <c r="L19" t="s">
         <v>8</v>
       </c>
-      <c r="L19">
+      <c r="M19">
         <v>1.06</v>
       </c>
-      <c r="M19">
+      <c r="N19">
         <v>0.94</v>
       </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:14">
       <c r="A20" t="s">
         <v>54</v>
       </c>
-      <c r="B20">
-        <v>1</v>
-      </c>
       <c r="C20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -2620,119 +2626,119 @@
       <c r="F20">
         <v>0</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20" t="s">
         <v>77</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <v>1.0501068</v>
       </c>
-      <c r="I20">
+      <c r="J20">
         <v>-5.4100729000000003</v>
       </c>
-      <c r="J20">
+      <c r="K20">
         <v>345</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
         <v>76</v>
       </c>
-      <c r="L20">
+      <c r="M20">
         <v>1.06</v>
       </c>
-      <c r="M20">
+      <c r="N20">
         <v>0.94</v>
       </c>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:14">
       <c r="A21" t="s">
         <v>55</v>
       </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
       <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
         <v>680</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>103</v>
       </c>
-      <c r="E21">
-        <v>0</v>
-      </c>
       <c r="F21">
         <v>0</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21" t="s">
         <v>77</v>
       </c>
-      <c r="H21">
+      <c r="I21">
         <v>0.99101054</v>
       </c>
-      <c r="I21">
+      <c r="J21">
         <v>-6.8211782999999997</v>
       </c>
-      <c r="J21">
+      <c r="K21">
         <v>345</v>
       </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
         <v>76</v>
       </c>
-      <c r="L21">
+      <c r="M21">
         <v>1.06</v>
       </c>
-      <c r="M21">
+      <c r="N21">
         <v>0.94</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:14">
       <c r="A22" t="s">
         <v>56</v>
       </c>
-      <c r="B22">
-        <v>1</v>
-      </c>
       <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
         <v>274</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>115</v>
       </c>
-      <c r="E22">
-        <v>0</v>
-      </c>
       <c r="F22">
         <v>0</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22" t="s">
         <v>77</v>
       </c>
-      <c r="H22">
+      <c r="I22">
         <v>1.0323192000000001</v>
       </c>
-      <c r="I22">
+      <c r="J22">
         <v>-7.6287460999999999</v>
       </c>
-      <c r="J22">
+      <c r="K22">
         <v>345</v>
       </c>
-      <c r="K22" t="s">
+      <c r="L22" t="s">
         <v>76</v>
       </c>
-      <c r="L22">
+      <c r="M22">
         <v>1.06</v>
       </c>
-      <c r="M22">
+      <c r="N22">
         <v>0.94</v>
       </c>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:14">
       <c r="A23" t="s">
         <v>57</v>
       </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
       <c r="C23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -2743,325 +2749,325 @@
       <c r="F23">
         <v>0</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23" t="s">
         <v>77</v>
       </c>
-      <c r="H23">
+      <c r="I23">
         <v>1.0501427000000001</v>
       </c>
-      <c r="I23">
+      <c r="J23">
         <v>-3.1831198999999999</v>
       </c>
-      <c r="J23">
+      <c r="K23">
         <v>345</v>
       </c>
-      <c r="K23" t="s">
+      <c r="L23" t="s">
         <v>76</v>
       </c>
-      <c r="L23">
+      <c r="M23">
         <v>1.06</v>
       </c>
-      <c r="M23">
+      <c r="N23">
         <v>0.94</v>
       </c>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:14">
       <c r="A24" t="s">
         <v>58</v>
       </c>
-      <c r="B24">
-        <v>1</v>
-      </c>
       <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
         <v>247.5</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>84.6</v>
       </c>
-      <c r="E24">
-        <v>0</v>
-      </c>
       <c r="F24">
         <v>0</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24" t="s">
         <v>77</v>
       </c>
-      <c r="H24">
+      <c r="I24">
         <v>1.0451451</v>
       </c>
-      <c r="I24">
+      <c r="J24">
         <v>-3.3812763000000001</v>
       </c>
-      <c r="J24">
+      <c r="K24">
         <v>345</v>
       </c>
-      <c r="K24" t="s">
+      <c r="L24" t="s">
         <v>76</v>
       </c>
-      <c r="L24">
+      <c r="M24">
         <v>1.06</v>
       </c>
-      <c r="M24">
+      <c r="N24">
         <v>0.94</v>
       </c>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:14">
       <c r="A25" t="s">
         <v>59</v>
       </c>
-      <c r="B25">
-        <v>1</v>
-      </c>
       <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
         <v>308.60000000000002</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>-92.2</v>
       </c>
-      <c r="E25">
-        <v>0</v>
-      </c>
       <c r="F25">
         <v>0</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25" t="s">
         <v>77</v>
       </c>
-      <c r="H25">
+      <c r="I25">
         <v>1.038001</v>
       </c>
-      <c r="I25">
+      <c r="J25">
         <v>-9.9137585000000001</v>
       </c>
-      <c r="J25">
+      <c r="K25">
         <v>345</v>
       </c>
-      <c r="K25" t="s">
+      <c r="L25" t="s">
         <v>76</v>
       </c>
-      <c r="L25">
+      <c r="M25">
         <v>1.06</v>
       </c>
-      <c r="M25">
+      <c r="N25">
         <v>0.94</v>
       </c>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:14">
       <c r="A26" t="s">
         <v>60</v>
       </c>
-      <c r="B26">
-        <v>1</v>
-      </c>
       <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
         <v>224</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <v>47.2</v>
       </c>
-      <c r="E26">
-        <v>0</v>
-      </c>
       <c r="F26">
         <v>0</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26" t="s">
         <v>77</v>
       </c>
-      <c r="H26">
+      <c r="I26">
         <v>1.0576827</v>
       </c>
-      <c r="I26">
+      <c r="J26">
         <v>-8.3692354000000009</v>
       </c>
-      <c r="J26">
+      <c r="K26">
         <v>345</v>
       </c>
-      <c r="K26" t="s">
+      <c r="L26" t="s">
         <v>8</v>
       </c>
-      <c r="L26">
+      <c r="M26">
         <v>1.06</v>
       </c>
-      <c r="M26">
+      <c r="N26">
         <v>0.94</v>
       </c>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:14">
       <c r="A27" t="s">
         <v>61</v>
       </c>
-      <c r="B27">
-        <v>1</v>
-      </c>
       <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
         <v>139</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <v>17</v>
       </c>
-      <c r="E27">
-        <v>0</v>
-      </c>
       <c r="F27">
         <v>0</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27" t="s">
         <v>77</v>
       </c>
-      <c r="H27">
+      <c r="I27">
         <v>1.0525613</v>
       </c>
-      <c r="I27">
+      <c r="J27">
         <v>-9.4387696000000005</v>
       </c>
-      <c r="J27">
+      <c r="K27">
         <v>345</v>
       </c>
-      <c r="K27" t="s">
+      <c r="L27" t="s">
         <v>8</v>
       </c>
-      <c r="L27">
+      <c r="M27">
         <v>1.06</v>
       </c>
-      <c r="M27">
+      <c r="N27">
         <v>0.94</v>
       </c>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:14">
       <c r="A28" t="s">
         <v>62</v>
       </c>
-      <c r="B28">
-        <v>1</v>
-      </c>
       <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
         <v>281</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <v>75.5</v>
       </c>
-      <c r="E28">
-        <v>0</v>
-      </c>
       <c r="F28">
         <v>0</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28" t="s">
         <v>77</v>
       </c>
-      <c r="H28">
+      <c r="I28">
         <v>1.0383449</v>
       </c>
-      <c r="I28">
+      <c r="J28">
         <v>-11.362152</v>
       </c>
-      <c r="J28">
+      <c r="K28">
         <v>345</v>
       </c>
-      <c r="K28" t="s">
+      <c r="L28" t="s">
         <v>8</v>
       </c>
-      <c r="L28">
+      <c r="M28">
         <v>1.06</v>
       </c>
-      <c r="M28">
+      <c r="N28">
         <v>0.94</v>
       </c>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:14">
       <c r="A29" t="s">
         <v>63</v>
       </c>
-      <c r="B29">
-        <v>1</v>
-      </c>
       <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29">
         <v>206</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <v>27.6</v>
       </c>
-      <c r="E29">
-        <v>0</v>
-      </c>
       <c r="F29">
         <v>0</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29" t="s">
         <v>77</v>
       </c>
-      <c r="H29">
+      <c r="I29">
         <v>1.0503737</v>
       </c>
-      <c r="I29">
+      <c r="J29">
         <v>-5.9283592000000001</v>
       </c>
-      <c r="J29">
+      <c r="K29">
         <v>345</v>
       </c>
-      <c r="K29" t="s">
+      <c r="L29" t="s">
         <v>76</v>
       </c>
-      <c r="L29">
+      <c r="M29">
         <v>1.06</v>
       </c>
-      <c r="M29">
+      <c r="N29">
         <v>0.94</v>
       </c>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:14">
       <c r="A30" t="s">
         <v>64</v>
       </c>
-      <c r="B30">
-        <v>1</v>
-      </c>
       <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30">
         <v>283.5</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <v>26.9</v>
       </c>
-      <c r="E30">
-        <v>0</v>
-      </c>
       <c r="F30">
         <v>0</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30" t="s">
         <v>77</v>
       </c>
-      <c r="H30">
+      <c r="I30">
         <v>1.0501149000000001</v>
       </c>
-      <c r="I30">
+      <c r="J30">
         <v>-3.1698740999999999</v>
       </c>
-      <c r="J30">
+      <c r="K30">
         <v>345</v>
       </c>
-      <c r="K30" t="s">
+      <c r="L30" t="s">
         <v>76</v>
       </c>
-      <c r="L30">
+      <c r="M30">
         <v>1.06</v>
       </c>
-      <c r="M30">
+      <c r="N30">
         <v>0.94</v>
       </c>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:14">
       <c r="A31" t="s">
         <v>65</v>
       </c>
-      <c r="B31">
+      <c r="C31">
         <v>2</v>
       </c>
-      <c r="C31">
-        <v>0</v>
-      </c>
       <c r="D31">
         <v>0</v>
       </c>
@@ -3071,79 +3077,79 @@
       <c r="F31">
         <v>0</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31" t="s">
         <v>77</v>
       </c>
-      <c r="H31">
+      <c r="I31">
         <v>1.0499000000000001</v>
       </c>
-      <c r="I31">
+      <c r="J31">
         <v>-7.3704745999999997</v>
       </c>
-      <c r="J31">
+      <c r="K31">
         <v>345</v>
       </c>
-      <c r="K31" t="s">
+      <c r="L31" t="s">
         <v>8</v>
       </c>
-      <c r="L31">
+      <c r="M31">
         <v>1.06</v>
       </c>
-      <c r="M31">
+      <c r="N31">
         <v>0.94</v>
       </c>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:14">
       <c r="A32" t="s">
         <v>66</v>
       </c>
-      <c r="B32">
+      <c r="C32">
         <v>3</v>
       </c>
-      <c r="C32">
+      <c r="D32">
         <v>9.1999999999999993</v>
       </c>
-      <c r="D32">
+      <c r="E32">
         <v>4.5999999999999996</v>
       </c>
-      <c r="E32">
-        <v>0</v>
-      </c>
       <c r="F32">
         <v>0</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32" t="s">
         <v>77</v>
       </c>
-      <c r="H32">
+      <c r="I32">
         <v>0.98199999999999998</v>
       </c>
-      <c r="I32">
-        <v>0</v>
-      </c>
       <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32">
         <v>345</v>
       </c>
-      <c r="K32" t="s">
+      <c r="L32" t="s">
         <v>75</v>
       </c>
-      <c r="L32">
+      <c r="M32">
         <v>1.06</v>
       </c>
-      <c r="M32">
+      <c r="N32">
         <v>0.94</v>
       </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:14">
       <c r="A33" t="s">
         <v>67</v>
       </c>
-      <c r="B33">
+      <c r="C33">
         <v>2</v>
       </c>
-      <c r="C33">
-        <v>0</v>
-      </c>
       <c r="D33">
         <v>0</v>
       </c>
@@ -3153,38 +3159,38 @@
       <c r="F33">
         <v>0</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G33">
+        <v>0</v>
+      </c>
+      <c r="H33" t="s">
         <v>77</v>
       </c>
-      <c r="H33">
+      <c r="I33">
         <v>0.98409999999999997</v>
       </c>
-      <c r="I33">
+      <c r="J33">
         <v>-0.1884374</v>
       </c>
-      <c r="J33">
+      <c r="K33">
         <v>345</v>
       </c>
-      <c r="K33" t="s">
+      <c r="L33" t="s">
         <v>75</v>
       </c>
-      <c r="L33">
+      <c r="M33">
         <v>1.06</v>
       </c>
-      <c r="M33">
+      <c r="N33">
         <v>0.94</v>
       </c>
     </row>
-    <row r="34" spans="1:13">
+    <row r="34" spans="1:14">
       <c r="A34" t="s">
         <v>68</v>
       </c>
-      <c r="B34">
+      <c r="C34">
         <v>2</v>
       </c>
-      <c r="C34">
-        <v>0</v>
-      </c>
       <c r="D34">
         <v>0</v>
       </c>
@@ -3194,38 +3200,38 @@
       <c r="F34">
         <v>0</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34" t="s">
         <v>77</v>
       </c>
-      <c r="H34">
+      <c r="I34">
         <v>0.99719999999999998</v>
       </c>
-      <c r="I34">
+      <c r="J34">
         <v>-0.19317445</v>
       </c>
-      <c r="J34">
+      <c r="K34">
         <v>345</v>
       </c>
-      <c r="K34" t="s">
+      <c r="L34" t="s">
         <v>76</v>
       </c>
-      <c r="L34">
+      <c r="M34">
         <v>1.06</v>
       </c>
-      <c r="M34">
+      <c r="N34">
         <v>0.94</v>
       </c>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:14">
       <c r="A35" t="s">
         <v>69</v>
       </c>
-      <c r="B35">
+      <c r="C35">
         <v>2</v>
       </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
       <c r="D35">
         <v>0</v>
       </c>
@@ -3235,38 +3241,38 @@
       <c r="F35">
         <v>0</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G35">
+        <v>0</v>
+      </c>
+      <c r="H35" t="s">
         <v>77</v>
       </c>
-      <c r="H35">
+      <c r="I35">
         <v>1.0123</v>
       </c>
-      <c r="I35">
+      <c r="J35">
         <v>-1.631119</v>
       </c>
-      <c r="J35">
+      <c r="K35">
         <v>345</v>
       </c>
-      <c r="K35" t="s">
+      <c r="L35" t="s">
         <v>76</v>
       </c>
-      <c r="L35">
+      <c r="M35">
         <v>1.06</v>
       </c>
-      <c r="M35">
+      <c r="N35">
         <v>0.94</v>
       </c>
     </row>
-    <row r="36" spans="1:13">
+    <row r="36" spans="1:14">
       <c r="A36" t="s">
         <v>70</v>
       </c>
-      <c r="B36">
+      <c r="C36">
         <v>2</v>
       </c>
-      <c r="C36">
-        <v>0</v>
-      </c>
       <c r="D36">
         <v>0</v>
       </c>
@@ -3276,38 +3282,38 @@
       <c r="F36">
         <v>0</v>
       </c>
-      <c r="G36" t="s">
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36" t="s">
         <v>77</v>
       </c>
-      <c r="H36">
+      <c r="I36">
         <v>1.0494000000000001</v>
       </c>
-      <c r="I36">
+      <c r="J36">
         <v>1.7765069</v>
       </c>
-      <c r="J36">
+      <c r="K36">
         <v>345</v>
       </c>
-      <c r="K36" t="s">
+      <c r="L36" t="s">
         <v>76</v>
       </c>
-      <c r="L36">
+      <c r="M36">
         <v>1.06</v>
       </c>
-      <c r="M36">
+      <c r="N36">
         <v>0.94</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:14">
       <c r="A37" t="s">
         <v>71</v>
       </c>
-      <c r="B37">
+      <c r="C37">
         <v>2</v>
       </c>
-      <c r="C37">
-        <v>0</v>
-      </c>
       <c r="D37">
         <v>0</v>
       </c>
@@ -3317,38 +3323,38 @@
       <c r="F37">
         <v>0</v>
       </c>
-      <c r="G37" t="s">
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37" t="s">
         <v>77</v>
       </c>
-      <c r="H37">
+      <c r="I37">
         <v>1.0636000000000001</v>
       </c>
-      <c r="I37">
+      <c r="J37">
         <v>4.4684374</v>
       </c>
-      <c r="J37">
+      <c r="K37">
         <v>345</v>
       </c>
-      <c r="K37" t="s">
+      <c r="L37" t="s">
         <v>76</v>
       </c>
-      <c r="L37">
+      <c r="M37">
         <v>1.06</v>
       </c>
-      <c r="M37">
+      <c r="N37">
         <v>0.94</v>
       </c>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:14">
       <c r="A38" t="s">
         <v>72</v>
       </c>
-      <c r="B38">
+      <c r="C38">
         <v>2</v>
       </c>
-      <c r="C38">
-        <v>0</v>
-      </c>
       <c r="D38">
         <v>0</v>
       </c>
@@ -3358,38 +3364,38 @@
       <c r="F38">
         <v>0</v>
       </c>
-      <c r="G38" t="s">
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38" t="s">
         <v>77</v>
       </c>
-      <c r="H38">
+      <c r="I38">
         <v>1.0275000000000001</v>
       </c>
-      <c r="I38">
+      <c r="J38">
         <v>-1.5828987999999999</v>
       </c>
-      <c r="J38">
+      <c r="K38">
         <v>345</v>
       </c>
-      <c r="K38" t="s">
+      <c r="L38" t="s">
         <v>8</v>
       </c>
-      <c r="L38">
+      <c r="M38">
         <v>1.06</v>
       </c>
-      <c r="M38">
+      <c r="N38">
         <v>0.94</v>
       </c>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:14">
       <c r="A39" t="s">
         <v>73</v>
       </c>
-      <c r="B39">
+      <c r="C39">
         <v>2</v>
       </c>
-      <c r="C39">
-        <v>0</v>
-      </c>
       <c r="D39">
         <v>0</v>
       </c>
@@ -3399,66 +3405,69 @@
       <c r="F39">
         <v>0</v>
       </c>
-      <c r="G39" t="s">
+      <c r="G39">
+        <v>0</v>
+      </c>
+      <c r="H39" t="s">
         <v>77</v>
       </c>
-      <c r="H39">
+      <c r="I39">
         <v>1.0265</v>
       </c>
-      <c r="I39">
+      <c r="J39">
         <v>3.8928177000000002</v>
       </c>
-      <c r="J39">
+      <c r="K39">
         <v>345</v>
       </c>
-      <c r="K39" t="s">
+      <c r="L39" t="s">
         <v>76</v>
       </c>
-      <c r="L39">
+      <c r="M39">
         <v>1.06</v>
       </c>
-      <c r="M39">
+      <c r="N39">
         <v>0.94</v>
       </c>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:14">
       <c r="A40" t="s">
         <v>74</v>
       </c>
-      <c r="B40">
+      <c r="C40">
         <v>2</v>
       </c>
-      <c r="C40">
+      <c r="D40">
         <v>1104</v>
       </c>
-      <c r="D40">
+      <c r="E40">
         <v>250</v>
       </c>
-      <c r="E40">
-        <v>0</v>
-      </c>
       <c r="F40">
         <v>0</v>
       </c>
-      <c r="G40" t="s">
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40" t="s">
         <v>77</v>
       </c>
-      <c r="H40">
+      <c r="I40">
         <v>1.03</v>
       </c>
-      <c r="I40">
+      <c r="J40">
         <v>-14.535256</v>
       </c>
-      <c r="J40">
+      <c r="K40">
         <v>345</v>
       </c>
-      <c r="K40" t="s">
+      <c r="L40" t="s">
         <v>75</v>
       </c>
-      <c r="L40">
+      <c r="M40">
         <v>1.06</v>
       </c>
-      <c r="M40">
+      <c r="N40">
         <v>0.94</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add plotting functionality, island detection and fixes issue #48 and #49 (#50)
* add plotting functionality, island detection and fixes issue #48 and 49

* Just retain the test file results
</commit_message>
<xml_diff>
--- a/test/inputs/case39/case39.xlsx
+++ b/test/inputs/case39/case39.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nomyk\Desktop\Network Reduction Model\NetworkReduction.jl\test\inputs\case39\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{254E094D-4C92-47F4-B2DD-094E93ABDAC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC762E08-7933-4D41-BE06-667FEB243A30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lines" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="79">
   <si>
     <t>Line_name</t>
   </si>
@@ -262,6 +262,9 @@
   </si>
   <si>
     <t>Z</t>
+  </si>
+  <si>
+    <t>IsRepresentative</t>
   </si>
 </sst>
 </file>
@@ -1813,106 +1816,109 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E83B6B-55F4-43BC-99E9-09E10DB244FC}">
-  <dimension ref="A1:O40"/>
+  <dimension ref="A1:P40"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="15.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:16">
       <c r="A1" s="9" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="N1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="P1" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:16">
       <c r="A2" t="s">
         <v>36</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
       <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
         <v>97.6</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>44.2</v>
       </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
       <c r="F2">
         <v>0</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
         <v>77</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>1.0393836000000001</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>-13.536602</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>345</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>75</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>1.06</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>0.94</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:16">
       <c r="A3" t="s">
         <v>37</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
       <c r="C3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -1923,119 +1929,119 @@
       <c r="F3">
         <v>0</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
         <v>77</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>1.0484941000000001</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>-9.7852665999999999</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>345</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>75</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>1.06</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>0.94</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:16">
       <c r="A4" t="s">
         <v>38</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
       <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
         <v>322</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>2.4</v>
       </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
       <c r="F4">
         <v>0</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s">
         <v>77</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>1.0307077</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>-12.276384</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>345</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>8</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>1.06</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>0.94</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:16">
       <c r="A5" t="s">
         <v>39</v>
       </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
       <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
         <v>500</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>184</v>
       </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
       <c r="F5">
         <v>0</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="s">
         <v>77</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>1.0044599999999999</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>-12.626734000000001</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>345</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>8</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <v>1.06</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>0.94</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:16">
       <c r="A6" t="s">
         <v>40</v>
       </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
       <c r="C6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -2046,37 +2052,37 @@
       <c r="F6">
         <v>0</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
         <v>77</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>1.0060062999999999</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>-11.192339</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>345</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>8</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>1.06</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>0.94</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:16">
       <c r="A7" t="s">
         <v>41</v>
       </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
       <c r="C7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -2087,160 +2093,160 @@
       <c r="F7">
         <v>0</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
         <v>77</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>1.0082256000000001</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>-10.408329999999999</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>345</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>75</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>1.06</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>0.94</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:16">
       <c r="A8" t="s">
         <v>42</v>
       </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
       <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
         <v>233.8</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>84</v>
       </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
       <c r="F8">
         <v>0</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
         <v>77</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>0.99839728000000005</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>-12.755625999999999</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>345</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>75</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <v>1.06</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>0.94</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:16">
       <c r="A9" t="s">
         <v>43</v>
       </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
       <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
         <v>522</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>176.6</v>
       </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
       <c r="F9">
         <v>0</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
         <v>77</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>0.99787232000000003</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>-13.335844</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>345</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>75</v>
       </c>
-      <c r="L9">
+      <c r="M9">
         <v>1.06</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>0.94</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:16">
       <c r="A10" t="s">
         <v>44</v>
       </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
       <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
         <v>6.5</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>-66.599999999999994</v>
       </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
       <c r="F10">
         <v>0</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" t="s">
         <v>77</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>1.038332</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>-14.178442</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>345</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>75</v>
       </c>
-      <c r="L10">
+      <c r="M10">
         <v>1.06</v>
       </c>
-      <c r="M10">
+      <c r="N10">
         <v>0.94</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:16">
       <c r="A11" t="s">
         <v>45</v>
       </c>
-      <c r="B11">
-        <v>1</v>
-      </c>
       <c r="C11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -2251,37 +2257,37 @@
       <c r="F11">
         <v>0</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
         <v>77</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>1.0178430999999999</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>-8.1708750000000006</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>345</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>75</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <v>1.06</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <v>0.94</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:16">
       <c r="A12" t="s">
         <v>46</v>
       </c>
-      <c r="B12">
-        <v>1</v>
-      </c>
       <c r="C12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -2292,78 +2298,78 @@
       <c r="F12">
         <v>0</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12" t="s">
         <v>77</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>1.0133858</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>-8.9369662999999999</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>345</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>75</v>
       </c>
-      <c r="L12">
+      <c r="M12">
         <v>1.06</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <v>0.94</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:16">
       <c r="A13" t="s">
         <v>47</v>
       </c>
-      <c r="B13">
-        <v>1</v>
-      </c>
       <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
         <v>8.5299999999999994</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>88</v>
       </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
       <c r="F13">
         <v>0</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13" t="s">
         <v>77</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>1.000815</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>-8.9988235999999997</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>345</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>75</v>
       </c>
-      <c r="L13">
+      <c r="M13">
         <v>1.06</v>
       </c>
-      <c r="M13">
+      <c r="N13">
         <v>0.94</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:16">
       <c r="A14" t="s">
         <v>48</v>
       </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
       <c r="C14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -2374,37 +2380,37 @@
       <c r="F14">
         <v>0</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14" t="s">
         <v>77</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>1.014923</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>-8.9299271999999998</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>345</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>75</v>
       </c>
-      <c r="L14">
+      <c r="M14">
         <v>1.06</v>
       </c>
-      <c r="M14">
+      <c r="N14">
         <v>0.94</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:16">
       <c r="A15" t="s">
         <v>49</v>
       </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
       <c r="C15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -2415,119 +2421,119 @@
       <c r="F15">
         <v>0</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15" t="s">
         <v>77</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <v>1.012319</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <v>-10.715294999999999</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>345</v>
       </c>
-      <c r="K15" t="s">
+      <c r="L15" t="s">
         <v>75</v>
       </c>
-      <c r="L15">
+      <c r="M15">
         <v>1.06</v>
       </c>
-      <c r="M15">
+      <c r="N15">
         <v>0.94</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:16">
       <c r="A16" t="s">
         <v>50</v>
       </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
       <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
         <v>320</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>153</v>
       </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
       <c r="F16">
         <v>0</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16" t="s">
         <v>77</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>1.0161853999999999</v>
       </c>
-      <c r="I16">
+      <c r="J16">
         <v>-11.345399</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>345</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>76</v>
       </c>
-      <c r="L16">
+      <c r="M16">
         <v>1.06</v>
       </c>
-      <c r="M16">
+      <c r="N16">
         <v>0.94</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:14">
       <c r="A17" t="s">
         <v>51</v>
       </c>
-      <c r="B17">
-        <v>1</v>
-      </c>
       <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
         <v>329</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>32.299999999999997</v>
       </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
       <c r="F17">
         <v>0</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17" t="s">
         <v>77</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <v>1.0325203000000001</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <v>-10.033348</v>
       </c>
-      <c r="J17">
+      <c r="K17">
         <v>345</v>
       </c>
-      <c r="K17" t="s">
+      <c r="L17" t="s">
         <v>76</v>
       </c>
-      <c r="L17">
+      <c r="M17">
         <v>1.06</v>
       </c>
-      <c r="M17">
+      <c r="N17">
         <v>0.94</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:14">
       <c r="A18" t="s">
         <v>52</v>
       </c>
-      <c r="B18">
-        <v>1</v>
-      </c>
       <c r="C18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -2538,78 +2544,78 @@
       <c r="F18">
         <v>0</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
         <v>77</v>
       </c>
-      <c r="H18">
+      <c r="I18">
         <v>1.0342365</v>
       </c>
-      <c r="I18">
+      <c r="J18">
         <v>-11.116436</v>
       </c>
-      <c r="J18">
+      <c r="K18">
         <v>345</v>
       </c>
-      <c r="K18" t="s">
+      <c r="L18" t="s">
         <v>8</v>
       </c>
-      <c r="L18">
+      <c r="M18">
         <v>1.06</v>
       </c>
-      <c r="M18">
+      <c r="N18">
         <v>0.94</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:14">
       <c r="A19" t="s">
         <v>53</v>
       </c>
-      <c r="B19">
-        <v>1</v>
-      </c>
       <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
         <v>158</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>30</v>
       </c>
-      <c r="E19">
-        <v>0</v>
-      </c>
       <c r="F19">
         <v>0</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19" t="s">
         <v>77</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <v>1.0315726000000001</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <v>-11.986167999999999</v>
       </c>
-      <c r="J19">
+      <c r="K19">
         <v>345</v>
       </c>
-      <c r="K19" t="s">
+      <c r="L19" t="s">
         <v>8</v>
       </c>
-      <c r="L19">
+      <c r="M19">
         <v>1.06</v>
       </c>
-      <c r="M19">
+      <c r="N19">
         <v>0.94</v>
       </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:14">
       <c r="A20" t="s">
         <v>54</v>
       </c>
-      <c r="B20">
-        <v>1</v>
-      </c>
       <c r="C20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -2620,119 +2626,119 @@
       <c r="F20">
         <v>0</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20" t="s">
         <v>77</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <v>1.0501068</v>
       </c>
-      <c r="I20">
+      <c r="J20">
         <v>-5.4100729000000003</v>
       </c>
-      <c r="J20">
+      <c r="K20">
         <v>345</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
         <v>76</v>
       </c>
-      <c r="L20">
+      <c r="M20">
         <v>1.06</v>
       </c>
-      <c r="M20">
+      <c r="N20">
         <v>0.94</v>
       </c>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:14">
       <c r="A21" t="s">
         <v>55</v>
       </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
       <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
         <v>680</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>103</v>
       </c>
-      <c r="E21">
-        <v>0</v>
-      </c>
       <c r="F21">
         <v>0</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21" t="s">
         <v>77</v>
       </c>
-      <c r="H21">
+      <c r="I21">
         <v>0.99101054</v>
       </c>
-      <c r="I21">
+      <c r="J21">
         <v>-6.8211782999999997</v>
       </c>
-      <c r="J21">
+      <c r="K21">
         <v>345</v>
       </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
         <v>76</v>
       </c>
-      <c r="L21">
+      <c r="M21">
         <v>1.06</v>
       </c>
-      <c r="M21">
+      <c r="N21">
         <v>0.94</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:14">
       <c r="A22" t="s">
         <v>56</v>
       </c>
-      <c r="B22">
-        <v>1</v>
-      </c>
       <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
         <v>274</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>115</v>
       </c>
-      <c r="E22">
-        <v>0</v>
-      </c>
       <c r="F22">
         <v>0</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22" t="s">
         <v>77</v>
       </c>
-      <c r="H22">
+      <c r="I22">
         <v>1.0323192000000001</v>
       </c>
-      <c r="I22">
+      <c r="J22">
         <v>-7.6287460999999999</v>
       </c>
-      <c r="J22">
+      <c r="K22">
         <v>345</v>
       </c>
-      <c r="K22" t="s">
+      <c r="L22" t="s">
         <v>76</v>
       </c>
-      <c r="L22">
+      <c r="M22">
         <v>1.06</v>
       </c>
-      <c r="M22">
+      <c r="N22">
         <v>0.94</v>
       </c>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:14">
       <c r="A23" t="s">
         <v>57</v>
       </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
       <c r="C23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -2743,325 +2749,325 @@
       <c r="F23">
         <v>0</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23" t="s">
         <v>77</v>
       </c>
-      <c r="H23">
+      <c r="I23">
         <v>1.0501427000000001</v>
       </c>
-      <c r="I23">
+      <c r="J23">
         <v>-3.1831198999999999</v>
       </c>
-      <c r="J23">
+      <c r="K23">
         <v>345</v>
       </c>
-      <c r="K23" t="s">
+      <c r="L23" t="s">
         <v>76</v>
       </c>
-      <c r="L23">
+      <c r="M23">
         <v>1.06</v>
       </c>
-      <c r="M23">
+      <c r="N23">
         <v>0.94</v>
       </c>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:14">
       <c r="A24" t="s">
         <v>58</v>
       </c>
-      <c r="B24">
-        <v>1</v>
-      </c>
       <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
         <v>247.5</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>84.6</v>
       </c>
-      <c r="E24">
-        <v>0</v>
-      </c>
       <c r="F24">
         <v>0</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24" t="s">
         <v>77</v>
       </c>
-      <c r="H24">
+      <c r="I24">
         <v>1.0451451</v>
       </c>
-      <c r="I24">
+      <c r="J24">
         <v>-3.3812763000000001</v>
       </c>
-      <c r="J24">
+      <c r="K24">
         <v>345</v>
       </c>
-      <c r="K24" t="s">
+      <c r="L24" t="s">
         <v>76</v>
       </c>
-      <c r="L24">
+      <c r="M24">
         <v>1.06</v>
       </c>
-      <c r="M24">
+      <c r="N24">
         <v>0.94</v>
       </c>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:14">
       <c r="A25" t="s">
         <v>59</v>
       </c>
-      <c r="B25">
-        <v>1</v>
-      </c>
       <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
         <v>308.60000000000002</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>-92.2</v>
       </c>
-      <c r="E25">
-        <v>0</v>
-      </c>
       <c r="F25">
         <v>0</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25" t="s">
         <v>77</v>
       </c>
-      <c r="H25">
+      <c r="I25">
         <v>1.038001</v>
       </c>
-      <c r="I25">
+      <c r="J25">
         <v>-9.9137585000000001</v>
       </c>
-      <c r="J25">
+      <c r="K25">
         <v>345</v>
       </c>
-      <c r="K25" t="s">
+      <c r="L25" t="s">
         <v>76</v>
       </c>
-      <c r="L25">
+      <c r="M25">
         <v>1.06</v>
       </c>
-      <c r="M25">
+      <c r="N25">
         <v>0.94</v>
       </c>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:14">
       <c r="A26" t="s">
         <v>60</v>
       </c>
-      <c r="B26">
-        <v>1</v>
-      </c>
       <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
         <v>224</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <v>47.2</v>
       </c>
-      <c r="E26">
-        <v>0</v>
-      </c>
       <c r="F26">
         <v>0</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26" t="s">
         <v>77</v>
       </c>
-      <c r="H26">
+      <c r="I26">
         <v>1.0576827</v>
       </c>
-      <c r="I26">
+      <c r="J26">
         <v>-8.3692354000000009</v>
       </c>
-      <c r="J26">
+      <c r="K26">
         <v>345</v>
       </c>
-      <c r="K26" t="s">
+      <c r="L26" t="s">
         <v>8</v>
       </c>
-      <c r="L26">
+      <c r="M26">
         <v>1.06</v>
       </c>
-      <c r="M26">
+      <c r="N26">
         <v>0.94</v>
       </c>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:14">
       <c r="A27" t="s">
         <v>61</v>
       </c>
-      <c r="B27">
-        <v>1</v>
-      </c>
       <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
         <v>139</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <v>17</v>
       </c>
-      <c r="E27">
-        <v>0</v>
-      </c>
       <c r="F27">
         <v>0</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27" t="s">
         <v>77</v>
       </c>
-      <c r="H27">
+      <c r="I27">
         <v>1.0525613</v>
       </c>
-      <c r="I27">
+      <c r="J27">
         <v>-9.4387696000000005</v>
       </c>
-      <c r="J27">
+      <c r="K27">
         <v>345</v>
       </c>
-      <c r="K27" t="s">
+      <c r="L27" t="s">
         <v>8</v>
       </c>
-      <c r="L27">
+      <c r="M27">
         <v>1.06</v>
       </c>
-      <c r="M27">
+      <c r="N27">
         <v>0.94</v>
       </c>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:14">
       <c r="A28" t="s">
         <v>62</v>
       </c>
-      <c r="B28">
-        <v>1</v>
-      </c>
       <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
         <v>281</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <v>75.5</v>
       </c>
-      <c r="E28">
-        <v>0</v>
-      </c>
       <c r="F28">
         <v>0</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28" t="s">
         <v>77</v>
       </c>
-      <c r="H28">
+      <c r="I28">
         <v>1.0383449</v>
       </c>
-      <c r="I28">
+      <c r="J28">
         <v>-11.362152</v>
       </c>
-      <c r="J28">
+      <c r="K28">
         <v>345</v>
       </c>
-      <c r="K28" t="s">
+      <c r="L28" t="s">
         <v>8</v>
       </c>
-      <c r="L28">
+      <c r="M28">
         <v>1.06</v>
       </c>
-      <c r="M28">
+      <c r="N28">
         <v>0.94</v>
       </c>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:14">
       <c r="A29" t="s">
         <v>63</v>
       </c>
-      <c r="B29">
-        <v>1</v>
-      </c>
       <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29">
         <v>206</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <v>27.6</v>
       </c>
-      <c r="E29">
-        <v>0</v>
-      </c>
       <c r="F29">
         <v>0</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29" t="s">
         <v>77</v>
       </c>
-      <c r="H29">
+      <c r="I29">
         <v>1.0503737</v>
       </c>
-      <c r="I29">
+      <c r="J29">
         <v>-5.9283592000000001</v>
       </c>
-      <c r="J29">
+      <c r="K29">
         <v>345</v>
       </c>
-      <c r="K29" t="s">
+      <c r="L29" t="s">
         <v>76</v>
       </c>
-      <c r="L29">
+      <c r="M29">
         <v>1.06</v>
       </c>
-      <c r="M29">
+      <c r="N29">
         <v>0.94</v>
       </c>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:14">
       <c r="A30" t="s">
         <v>64</v>
       </c>
-      <c r="B30">
-        <v>1</v>
-      </c>
       <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30">
         <v>283.5</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <v>26.9</v>
       </c>
-      <c r="E30">
-        <v>0</v>
-      </c>
       <c r="F30">
         <v>0</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30" t="s">
         <v>77</v>
       </c>
-      <c r="H30">
+      <c r="I30">
         <v>1.0501149000000001</v>
       </c>
-      <c r="I30">
+      <c r="J30">
         <v>-3.1698740999999999</v>
       </c>
-      <c r="J30">
+      <c r="K30">
         <v>345</v>
       </c>
-      <c r="K30" t="s">
+      <c r="L30" t="s">
         <v>76</v>
       </c>
-      <c r="L30">
+      <c r="M30">
         <v>1.06</v>
       </c>
-      <c r="M30">
+      <c r="N30">
         <v>0.94</v>
       </c>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:14">
       <c r="A31" t="s">
         <v>65</v>
       </c>
-      <c r="B31">
+      <c r="C31">
         <v>2</v>
       </c>
-      <c r="C31">
-        <v>0</v>
-      </c>
       <c r="D31">
         <v>0</v>
       </c>
@@ -3071,79 +3077,79 @@
       <c r="F31">
         <v>0</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31" t="s">
         <v>77</v>
       </c>
-      <c r="H31">
+      <c r="I31">
         <v>1.0499000000000001</v>
       </c>
-      <c r="I31">
+      <c r="J31">
         <v>-7.3704745999999997</v>
       </c>
-      <c r="J31">
+      <c r="K31">
         <v>345</v>
       </c>
-      <c r="K31" t="s">
+      <c r="L31" t="s">
         <v>8</v>
       </c>
-      <c r="L31">
+      <c r="M31">
         <v>1.06</v>
       </c>
-      <c r="M31">
+      <c r="N31">
         <v>0.94</v>
       </c>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:14">
       <c r="A32" t="s">
         <v>66</v>
       </c>
-      <c r="B32">
+      <c r="C32">
         <v>3</v>
       </c>
-      <c r="C32">
+      <c r="D32">
         <v>9.1999999999999993</v>
       </c>
-      <c r="D32">
+      <c r="E32">
         <v>4.5999999999999996</v>
       </c>
-      <c r="E32">
-        <v>0</v>
-      </c>
       <c r="F32">
         <v>0</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32" t="s">
         <v>77</v>
       </c>
-      <c r="H32">
+      <c r="I32">
         <v>0.98199999999999998</v>
       </c>
-      <c r="I32">
-        <v>0</v>
-      </c>
       <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32">
         <v>345</v>
       </c>
-      <c r="K32" t="s">
+      <c r="L32" t="s">
         <v>75</v>
       </c>
-      <c r="L32">
+      <c r="M32">
         <v>1.06</v>
       </c>
-      <c r="M32">
+      <c r="N32">
         <v>0.94</v>
       </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:14">
       <c r="A33" t="s">
         <v>67</v>
       </c>
-      <c r="B33">
+      <c r="C33">
         <v>2</v>
       </c>
-      <c r="C33">
-        <v>0</v>
-      </c>
       <c r="D33">
         <v>0</v>
       </c>
@@ -3153,38 +3159,38 @@
       <c r="F33">
         <v>0</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G33">
+        <v>0</v>
+      </c>
+      <c r="H33" t="s">
         <v>77</v>
       </c>
-      <c r="H33">
+      <c r="I33">
         <v>0.98409999999999997</v>
       </c>
-      <c r="I33">
+      <c r="J33">
         <v>-0.1884374</v>
       </c>
-      <c r="J33">
+      <c r="K33">
         <v>345</v>
       </c>
-      <c r="K33" t="s">
+      <c r="L33" t="s">
         <v>75</v>
       </c>
-      <c r="L33">
+      <c r="M33">
         <v>1.06</v>
       </c>
-      <c r="M33">
+      <c r="N33">
         <v>0.94</v>
       </c>
     </row>
-    <row r="34" spans="1:13">
+    <row r="34" spans="1:14">
       <c r="A34" t="s">
         <v>68</v>
       </c>
-      <c r="B34">
+      <c r="C34">
         <v>2</v>
       </c>
-      <c r="C34">
-        <v>0</v>
-      </c>
       <c r="D34">
         <v>0</v>
       </c>
@@ -3194,38 +3200,38 @@
       <c r="F34">
         <v>0</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34" t="s">
         <v>77</v>
       </c>
-      <c r="H34">
+      <c r="I34">
         <v>0.99719999999999998</v>
       </c>
-      <c r="I34">
+      <c r="J34">
         <v>-0.19317445</v>
       </c>
-      <c r="J34">
+      <c r="K34">
         <v>345</v>
       </c>
-      <c r="K34" t="s">
+      <c r="L34" t="s">
         <v>76</v>
       </c>
-      <c r="L34">
+      <c r="M34">
         <v>1.06</v>
       </c>
-      <c r="M34">
+      <c r="N34">
         <v>0.94</v>
       </c>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:14">
       <c r="A35" t="s">
         <v>69</v>
       </c>
-      <c r="B35">
+      <c r="C35">
         <v>2</v>
       </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
       <c r="D35">
         <v>0</v>
       </c>
@@ -3235,38 +3241,38 @@
       <c r="F35">
         <v>0</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G35">
+        <v>0</v>
+      </c>
+      <c r="H35" t="s">
         <v>77</v>
       </c>
-      <c r="H35">
+      <c r="I35">
         <v>1.0123</v>
       </c>
-      <c r="I35">
+      <c r="J35">
         <v>-1.631119</v>
       </c>
-      <c r="J35">
+      <c r="K35">
         <v>345</v>
       </c>
-      <c r="K35" t="s">
+      <c r="L35" t="s">
         <v>76</v>
       </c>
-      <c r="L35">
+      <c r="M35">
         <v>1.06</v>
       </c>
-      <c r="M35">
+      <c r="N35">
         <v>0.94</v>
       </c>
     </row>
-    <row r="36" spans="1:13">
+    <row r="36" spans="1:14">
       <c r="A36" t="s">
         <v>70</v>
       </c>
-      <c r="B36">
+      <c r="C36">
         <v>2</v>
       </c>
-      <c r="C36">
-        <v>0</v>
-      </c>
       <c r="D36">
         <v>0</v>
       </c>
@@ -3276,38 +3282,38 @@
       <c r="F36">
         <v>0</v>
       </c>
-      <c r="G36" t="s">
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36" t="s">
         <v>77</v>
       </c>
-      <c r="H36">
+      <c r="I36">
         <v>1.0494000000000001</v>
       </c>
-      <c r="I36">
+      <c r="J36">
         <v>1.7765069</v>
       </c>
-      <c r="J36">
+      <c r="K36">
         <v>345</v>
       </c>
-      <c r="K36" t="s">
+      <c r="L36" t="s">
         <v>76</v>
       </c>
-      <c r="L36">
+      <c r="M36">
         <v>1.06</v>
       </c>
-      <c r="M36">
+      <c r="N36">
         <v>0.94</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:14">
       <c r="A37" t="s">
         <v>71</v>
       </c>
-      <c r="B37">
+      <c r="C37">
         <v>2</v>
       </c>
-      <c r="C37">
-        <v>0</v>
-      </c>
       <c r="D37">
         <v>0</v>
       </c>
@@ -3317,38 +3323,38 @@
       <c r="F37">
         <v>0</v>
       </c>
-      <c r="G37" t="s">
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37" t="s">
         <v>77</v>
       </c>
-      <c r="H37">
+      <c r="I37">
         <v>1.0636000000000001</v>
       </c>
-      <c r="I37">
+      <c r="J37">
         <v>4.4684374</v>
       </c>
-      <c r="J37">
+      <c r="K37">
         <v>345</v>
       </c>
-      <c r="K37" t="s">
+      <c r="L37" t="s">
         <v>76</v>
       </c>
-      <c r="L37">
+      <c r="M37">
         <v>1.06</v>
       </c>
-      <c r="M37">
+      <c r="N37">
         <v>0.94</v>
       </c>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:14">
       <c r="A38" t="s">
         <v>72</v>
       </c>
-      <c r="B38">
+      <c r="C38">
         <v>2</v>
       </c>
-      <c r="C38">
-        <v>0</v>
-      </c>
       <c r="D38">
         <v>0</v>
       </c>
@@ -3358,38 +3364,38 @@
       <c r="F38">
         <v>0</v>
       </c>
-      <c r="G38" t="s">
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38" t="s">
         <v>77</v>
       </c>
-      <c r="H38">
+      <c r="I38">
         <v>1.0275000000000001</v>
       </c>
-      <c r="I38">
+      <c r="J38">
         <v>-1.5828987999999999</v>
       </c>
-      <c r="J38">
+      <c r="K38">
         <v>345</v>
       </c>
-      <c r="K38" t="s">
+      <c r="L38" t="s">
         <v>8</v>
       </c>
-      <c r="L38">
+      <c r="M38">
         <v>1.06</v>
       </c>
-      <c r="M38">
+      <c r="N38">
         <v>0.94</v>
       </c>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:14">
       <c r="A39" t="s">
         <v>73</v>
       </c>
-      <c r="B39">
+      <c r="C39">
         <v>2</v>
       </c>
-      <c r="C39">
-        <v>0</v>
-      </c>
       <c r="D39">
         <v>0</v>
       </c>
@@ -3399,66 +3405,69 @@
       <c r="F39">
         <v>0</v>
       </c>
-      <c r="G39" t="s">
+      <c r="G39">
+        <v>0</v>
+      </c>
+      <c r="H39" t="s">
         <v>77</v>
       </c>
-      <c r="H39">
+      <c r="I39">
         <v>1.0265</v>
       </c>
-      <c r="I39">
+      <c r="J39">
         <v>3.8928177000000002</v>
       </c>
-      <c r="J39">
+      <c r="K39">
         <v>345</v>
       </c>
-      <c r="K39" t="s">
+      <c r="L39" t="s">
         <v>76</v>
       </c>
-      <c r="L39">
+      <c r="M39">
         <v>1.06</v>
       </c>
-      <c r="M39">
+      <c r="N39">
         <v>0.94</v>
       </c>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:14">
       <c r="A40" t="s">
         <v>74</v>
       </c>
-      <c r="B40">
+      <c r="C40">
         <v>2</v>
       </c>
-      <c r="C40">
+      <c r="D40">
         <v>1104</v>
       </c>
-      <c r="D40">
+      <c r="E40">
         <v>250</v>
       </c>
-      <c r="E40">
-        <v>0</v>
-      </c>
       <c r="F40">
         <v>0</v>
       </c>
-      <c r="G40" t="s">
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40" t="s">
         <v>77</v>
       </c>
-      <c r="H40">
+      <c r="I40">
         <v>1.03</v>
       </c>
-      <c r="I40">
+      <c r="J40">
         <v>-14.535256</v>
       </c>
-      <c r="J40">
+      <c r="K40">
         <v>345</v>
       </c>
-      <c r="K40" t="s">
+      <c r="L40" t="s">
         <v>75</v>
       </c>
-      <c r="L40">
+      <c r="M40">
         <v>1.06</v>
       </c>
-      <c r="M40">
+      <c r="N40">
         <v>0.94</v>
       </c>
     </row>

</xml_diff>